<commit_message>
docs: update GIM selection criteria spreadsheet
</commit_message>
<xml_diff>
--- a/docs/Критерии_отбора_ГИМ.xlsx
+++ b/docs/Критерии_отбора_ГИМ.xlsx
@@ -10,6 +10,7 @@
     <sheet name="5 Критериев отбора" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Объективные фильтры" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Направления ГИМ" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Паттерны кураторов 2024-2025" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -56,8 +57,14 @@
       <color rgb="00000000"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00595959"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -88,6 +95,12 @@
         <bgColor rgb="00C00000"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00203764"/>
+        <bgColor rgb="00203764"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -115,7 +128,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -141,6 +154,10 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -528,9 +545,9 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Разработано для QA/Бизнес-анализа (Issue #8) и контракта ИИ-оценщика (Issue #5). Версия от 21.10.2026</t>
+      <c r="A2" s="11" t="inlineStr">
+        <is>
+          <t>Обновлено по результатам глубокого анализа анкет 2024 (осень) и 2025 (весна) с оценками кураторов и данными активности. 21.10.2026</t>
         </is>
       </c>
     </row>
@@ -571,139 +588,147 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="110" customHeight="1">
+    <row r="5" ht="145" customHeight="1">
       <c r="A5" s="4" t="n">
         <v>1</v>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Мотивация и осознанность выбора</t>
+          <t>Мотивация и осознанность выбора
+(+ Сфера интересов и Источник прихода)</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
           <t>• Чёткие личные и профессиональные цели
-• Понимание музейной специфики
-• Интерес к истории и культуре
-• Знание о музее из надёжных источников (сайт, друзья, круглые столы)</t>
+• Осознанный источник прихода: личный поиск на сайте ГИМ, рекомендации действующих волонтёров, интерес к выставкам
+• Партнёрская мотивация («хочу помочь музею», «применить навыки для посетителей»)
+• Совпадение научных интересов с профилем ГИМ (археология, история России, архивы, музеология)
+• Фокус на 1–2 профильных направлениях</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>• Шаблонные отписки, общие фразы
-• Не объясняет выбор ГИМ
-• Жёсткая фиксация исключительно на фондовом направлении (риск «мёртвой души» при нехватке мест)
-• Интересы не связаны с музеем</t>
+          <t>• Административное принуждение от вуза («преподаватель сказал», «заставили в чате группы ради зачёта по практике») — главный триггер оценки 0 в 2025 г.!
+• Потребительская мотивация в 1–2 слова («Опыт», «Практика», «Интересно»)
+• Жёсткая фиксация исключительно на фондах («хочу только в фонд» — риск «мёртвой души»)
+• «Ковровый выбор» всех направлений подряд (все 5 галочек) без понимания их различий</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>• Анализ совпадения ценностей и ожиданий
-• Подсвечивание сильных цитат-обоснований
-• ❌ ЗАПРЕТ: не отказывать автоматически за лаконичность ответов</t>
+          <t>• Оценка глубины мотивации и искренности интереса
+• Фильтрация административно направленных студентов от мотивированных добровольцев
+• ❌ ЗАПРЕТ: не отказывать автоматически за лаконичность, если есть профильный интерес</t>
         </is>
       </c>
       <c r="F5" s="6" t="inlineStr">
         <is>
-          <t>«Мотивация: высокая / средняя / неясная»
-Цитата-обоснование из анкеты.
-Направленность интереса: карьерная / научная / социальная.</t>
+          <t>«Мотивация: высокая / средняя / формальная (риск принудительной практики)»
+Цитата-обоснование.
+Совпадение научных интересов с профилем музея: да / нет.</t>
         </is>
       </c>
       <c r="G5" s="6" t="inlineStr">
         <is>
-          <t>• Если выбраны только фонды: «Готовы ли вы помогать в других направлениях (медиа, проекты), если в фондах не будет мест?»
-• Если ответ краткий: «Что именно в Историческом музее вас больше всего привлекает?»</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="110" customHeight="1">
+          <t>• Если источник «ВУЗ/преподаватель»: «Что именно побудило вас подать заявку: личный интерес к истории или необходимость закрыть практику?»
+• Если выбраны все направления подряд: «Какое одно направление для вас действительно в приоритете и почему?»
+• Если ответ краткий: «Что конкретно в экспозиции ГИМ вам ближе всего?»</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="145" customHeight="1">
       <c r="A6" s="7" t="n">
         <v>2</v>
       </c>
       <c r="B6" s="8" t="inlineStr">
         <is>
-          <t>Опыт и навыки</t>
+          <t>Опыт и навыки
+(+ Софт-скиллы и «Суперсила»)</t>
         </is>
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>• Профильный опыт (музеи, выставки, архивы, экспедиции, инклюзия)
-• Прикладные навыки: фото, видео, монтаж, дизайн, тексты, ведение соцсетей
-• Языки B1+ (английский, китайский)
-• Опыт координации мероприятий</t>
+          <t>• Профильный опыт (музеи, выставки, архивы, археологические экспедиции, инклюзия)
+• Прикладные навыки: фото, видео, монтаж, дизайн, тексты, иностранные языки B1+
+• Опыт школьных/студенческих олимпиад («Музеи. Парки. Усадьбы», Всерос)
+• Осознанная «Суперсила» с привязкой к делу и самоиронией (усидчивость с документами, стрессоустойчивость, умение просто объяснять сложное)</t>
         </is>
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
-          <t>• Пустые графы в опыте
-• Не указано, чем конкретно кандидат хочет помочь музею
-• Непрофильное образование (лечфак, физика, инженерия — если нет пояснения)</t>
+          <t>• Пустые графы в опыте без попытки описать смежные навыки
+• Формализм в «Суперсиле»: прочерк, «не знаю», штампы («всегда встаю по утрам», «коммуникабельность» в 1 слово), пафосные цитаты без связи с задачами
+• Не указано, чем именно кандидат может быть полезен музею</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
         <is>
-          <t>• Мэтчинг компетенций под 5 направлений
-• ❌ ЗАПРЕТ: не снижать баллы за отсутствие профильного опыта или непрофильный вуз (музею нужны волонтёры самых разных профилей)</t>
+          <t>• Мэтчинг компетенций под направления музея
+• Анализ адекватности самооценки и софт-скиллов по ответу о суперсиле
+• ❌ ЗАПРЕТ: не отсекать кандидатов с непрофильным образованием (инженеры, медики) при наличии мотивации</t>
         </is>
       </c>
       <c r="F6" s="9" t="inlineStr">
         <is>
-          <t>«Подтверждённые навыки: [список]»
-«Рекомендованные направления: [направления]»
-«Профиль образования / работы».</t>
+          <t>«Подтверждённые hard skills: [список]»
+«Качество софт-скиллов (по суперсиле): зрелое / формальное»
+«Рекомендованные направления ГИМ».</t>
         </is>
       </c>
       <c r="G6" s="9" t="inlineStr">
         <is>
-          <t>• «Какие форматы мероприятий вам ближе: мастер-классы, квесты, экскурсии или сопровождение?»
-• Для медиа: «Есть ли примеры ваших видео/фото/текстов?»
-• «В чём именно хотели бы попрактиковаться?»</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="110" customHeight="1">
+          <t>• По суперсиле: «Приведите пример, когда ваша суперсила помогла решить сложную или нестандартную задачу?»
+• Для медиа/проектов: «Есть ли готовые примеры ваших текстов, фото, видео или сценариев мероприятий?»
+• «В чём именно вам хотелось бы попрактиковаться в ГИМ?»</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="145" customHeight="1">
       <c r="A7" s="4" t="n">
         <v>3</v>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Курс обучения и нагрузка</t>
+          <t>Курс обучения и нагрузка
+(+ Конфликт параллельных проектов)</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>• Старшие курсы (2+ курс бакалавриата, магистратура)
-• Оконченное образование / работа со стабильным графиком
-• Осознанное распределение времени</t>
+          <t>• Старшие курсы (2–4 курс бакалавриата, магистратура), выпускники со стабильным графиком
+• Наличие свободного времени в графике (выходные, будни вечер)
+• Реалистичное понимание объёма времени (от 16 часов в месяц)</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>• 1-й курс бакалавриата (статистический риск выгорания / перегрузки первой сессией)
-• Высокая загруженность (очная учёба + full-time работа)</t>
+          <t>• 1-й курс бакалавриата (статистический риск выгорания и завала первой сессии)
+• ⚠️ УЧАСТИЕ В ДРУГИХ СХОЖИХ ПРОЕКТАХ ПРЯМО СЕЙЧАС (волонтёрство в Третьяковке/Пушкинском, работа в другом музее, актив в студсовете одновременно) — риск распыления и нулевой выработки часов!
+• Высокая загруженность (очная учёба + full-time работа без гибкого графика)</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>• Оценка риска доступности по часам
-• ❌ СТРОГИЙ ЗАПРЕТ: не снижать оценку и не отсекать первокурсников автоматически! Это этический и продуктовый риск</t>
+          <t>• Индикация рисков доступности и конфликта расписаний
+• Подсвечивание маркера «Параллельные проекты / Мультизанятость»
+• ❌ СТРОГИЙ ЗАПРЕТ: не ставить автоматический отказ первокурсникам и занятым людям, а выносить вопрос о часах на интервью</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>«Маркер нагрузки: 1 курс / совмещение с работой»
-Рекомендация: обсудить на интервью график сессий и реалистичность выделения часов.</t>
+          <t>«Маркер нагрузки: 1 курс / совмещение с работой / параллельные проекты [указать какие]»
+Рекомендация: детально согласовать график дежурств и приоритет ГИМ на очном интервью.</t>
         </is>
       </c>
       <c r="G7" s="6" t="inlineStr">
         <is>
-          <t>• «Сколько часов в месяц вы реально готовы выделять (норма ~16 ч)?»
-• «Какой график вам удобнее: регулярные смены по выходным или проектное участие в разовых событиях?»</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="110" customHeight="1">
+          <t>• По параллельным проектам: «Вы указали участие в проекте [X]. Сколько конкретно часов в неделю вы сможете гарантированно уделять ГИМ без ущерба для текущих обязательств?»
+• «Какой график вам удобнее: регулярные дежурства по субботам/воскресеньям или разовые акции?»</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="145" customHeight="1">
       <c r="A8" s="7" t="n">
         <v>4</v>
       </c>
@@ -714,27 +739,28 @@
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>• Развёрнутая, структурированная анкета
-• Корректная работающая ссылка на страницу ВКонтакте для оперативной связи</t>
+          <t>• Развёрнутая, структурированная анкета с законченными мыслями
+• Корректная работающая ссылка на страницу ВКонтакте для оперативной связи
+• Открытый диалог при заполнении</t>
         </is>
       </c>
       <c r="D8" s="9" t="inlineStr">
         <is>
-          <t>• Полупустая или пустая анкета
-• Не указана страница ВК (только телефон)
-• Закрытый профиль ВК / пустая страница</t>
+          <t>• Полупустая анкета («телеграфный стиль», ответы по 1–2 слова)
+• Не указана ссылка на ВК (указан только телефон)
+• Закрытый профиль ВК / пустая страница без активности</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
         <is>
           <t>• Проверка полноты заполнения полей
-• Проверка наличия канала связи (ВК — основной канал музея)
-• ❌ ЗАПРЕТ: не парсить закрытые страницы и не штрафовать за настройки приватности профиля</t>
+• Верификация канала связи (ВК — основной рабочий инструмент музея)
+• ❌ ЗАПРЕТ: не парсить закрытые страницы и не снижать оценку за настройки приватности</t>
         </is>
       </c>
       <c r="F8" s="9" t="inlineStr">
         <is>
-          <t>«Полнота анкеты: высокая / средняя / низкая»
+          <t>«Полнота анкеты: высокая / средняя / низкая (телеграфный стиль)»
 «Статус канала связи: VK предоставлен / требуется подтвердить контакт».</t>
         </is>
       </c>
@@ -745,45 +771,47 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="110" customHeight="1">
+    <row r="9" ht="145" customHeight="1">
       <c r="A9" s="4" t="n">
         <v>5</v>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Логистика и бытовые вопросы</t>
+          <t>Логистика и бытовые вопросы
+(+ График музейных событий)</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
           <t>• Проживание в Москве или ближнем Подмосковье
-• Реалистичная оценка времени на дорогу
-• Готовность к очным сменам в музее</t>
+• Реалистичная оценка времени на дорогу до Красной площади
+• Готовность к очным сменам в дни проведения музейных мероприятий</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>• Проживание в других городах России (при выборе очных направлений)
-• Мультиволонтёрство: активное участие сразу в 3+ других волонтёрских организациях (риск нехватки времени)</t>
+          <t>• Проживание в других регионах России (при выборе очных направлений)
+• Несовместимость графика с днями ключевых акций музея (четверги/пятницы вечер, выходные дни)</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>• Проверка доступности для очных смен
-• ❌ ЗАПРЕТ: не отсекать иногородних студентов московских вузов и кандидатов на дистанционные задачи (медиа/тексты/переводы)</t>
+          <t>• Проверка территориальной доступности для очных смен
+• Маршрутизация иногородних на удалённые треки (медиа, тексты, дизайн)
+• ❌ ЗАПРЕТ: не отсекать иногородних студентов московских вузов</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
           <t>«Локация: Москва / Иногородний»
-«Формат участия: очный / возможен онлайн»
-«Риск мультиволонтёрства: да / нет».</t>
+«Формат участия: очный / возможен онлайн (медиа)»
+«Готовность к сменам в выходные дни».</t>
         </is>
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
           <t>• «Планируете ли вы очное участие в Москве или рассматриваете дистанционные задачи (медиа, переводы, тексты)?»
-• «Состоите ли вы сейчас в других волонтёрских программах?»</t>
+• «Удобно ли вам участвовать в мероприятиях по выходным и в вечернее время?»</t>
         </is>
       </c>
     </row>
@@ -1172,4 +1200,179 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Аналитический срез реальных анкет 2024–2025 гг. и решений кураторов ГИМ</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="11" t="inlineStr">
+        <is>
+          <t>Базируется на выборке из 180+ анкет (materials/gim): выявление ключевых драйверов высоких и низких оценок</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="28" customHeight="1">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>Категория анализа</t>
+        </is>
+      </c>
+      <c r="B4" s="12" t="inlineStr">
+        <is>
+          <t>Фактический паттерн из данных</t>
+        </is>
+      </c>
+      <c r="C4" s="12" t="inlineStr">
+        <is>
+          <t>Статистика / Примеры из таблиц</t>
+        </is>
+      </c>
+      <c r="D4" s="12" t="inlineStr">
+        <is>
+          <t>Вывод и рекомендация для нашего ИИ</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="110" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>1. Феномен оценки 0
+(Отказ без собеседования)</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>ВЕСНА 2025: 27 анкет получили 0 баллов из-за административного принуждения со стороны вуза (ГУП / МГОУ). Кандидатов обязали подать заявку ради учебной практики.</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Источник: «Сказали в чате группы», «Преподаватель», «Администрация вуза».
+Ожидания: «Опыт», «Пройти практику».
+Суперсила: «-», «Не знаю», «Всегда встаю по будильнику».</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>ИИ должен выявлять отсутствие личной мотивации и шаблонные отписки «для галочки». Задавать проверочный вопрос о личной цели участия.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="110" customHeight="1">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>2. Параллельные проекты
+(Риск мультизанятости)</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>Кандидаты, которые прямо сейчас волонтёрят в 2–3 музеях (Пушкинский, Третьяковка, Музей Москвы) или работают full-time, в 2024 г. показали выработку часов &lt; 10 ч/год или выбыли.</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>Примеры: волонтёр НИУ ВШЭ + Пушкинский + Третьяковка (активность 23 ч); работа в РГАЛИ + Artlife (активность снижена).
+У кандидата с 3 проектами активность = 0 ч.</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>Не отказывать автоматически, но маркировать как риск нехватки времени. ИИ генерирует вопрос о распределении часов между проектами.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="110" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>3. Портрет «Звёздного волонтёра»
+(Активность &gt; 30–300 часов)</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Студенты 2–4 курсов (РГГУ, МГУ, ВШЭ, МПГУ) или выпускники с профильным интересом к истории/музеологии, имеющие опыт олимпиад («Музеи. Парки. Усадьбы») или практики.</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>Рекордсмен 2024 г. (317 часов!): РГГУ, 3 курс, олимпиада «Музеи. Парки. Усадьбы», чёткое понимание специфики квестов и фондов, суперсила — стрессоустойчивость.</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>ИИ должен начислять повышенный скоринг за профильные олимпиады, конкретный фокус в направлениях и зрелую рефлексию.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="110" customHeight="1">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>4. Графа «Суперсила» как фильтр
+софт-скиллов</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>Кураторы используют ответ о суперсиле как маркер зрелости и чувства юмора. Успешные кандидаты пишут о прикладных софт-скиллах, отсеянные — ставят прочерк или банальность.</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>Балл 3: «Въедливость, могу долго сидеть над монотонной задачей», «Умею говорить забавным голосом и объяснять сложное просто».
+Балл 0: «-», «Коммуникабельность», «Вставать по утрам».</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>ИИ анализирует текстовое качество ответа на вопрос о суперсиле: содержательность, самоирония, прикладной характер для работы с людьми/экспонатами.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="110" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>5. «Ковровый выбор» направлений</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Кандидаты с баллом 0 и 1 почти всегда отмечают ВСЕ доступные направления подряд (Организация, Проекты, Фонды, Инклюзия).</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>В анкетах со Score 0: 4–5 направлений выбраны одновременно без единого комментария в опыте.
+В анкетах со Score 3: выбрано 1–2 сфокусированных трека.</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>ИИ детектирует выбор &gt;3 направлений как маркер неопределённости и формирует диалоговое уточнение: «Какое направление для вас ключевое?»</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
docs: update GIM selection criteria spreadsheet and gitignore
</commit_message>
<xml_diff>
--- a/docs/Критерии_отбора_ГИМ.xlsx
+++ b/docs/Критерии_отбора_ГИМ.xlsx
@@ -10,7 +10,7 @@
     <sheet name="5 Критериев отбора" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Объективные фильтры" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Направления ГИМ" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Паттерны кураторов 2024-2025" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Правила скрининга анкеты" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -38,7 +38,7 @@
       <name val="Calibri"/>
       <i val="1"/>
       <color rgb="00595959"/>
-      <sz val="11"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -55,12 +55,6 @@
     <font>
       <name val="Calibri"/>
       <color rgb="00000000"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <i val="1"/>
-      <color rgb="00595959"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -128,7 +122,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -156,7 +150,6 @@
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -529,9 +522,9 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
     <col width="32" customWidth="1" min="3" max="3"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
     <col width="34" customWidth="1" min="5" max="5"/>
     <col width="30" customWidth="1" min="6" max="6"/>
     <col width="36" customWidth="1" min="7" max="7"/>
@@ -540,18 +533,18 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Государственный исторический музей (ГИМ) · Матрица 5 критериев отбора волонтёров</t>
+          <t>Государственный исторический музей (ГИМ) · Критерии первичного скрининга анкеты</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="11" t="inlineStr">
-        <is>
-          <t>Обновлено по результатам глубокого анализа анкет 2024 (осень) и 2025 (весна) с оценками кураторов и данными активности. 21.10.2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="28" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Фокус: автоматическая фильтрация и выявление рисков на этапе входной анкеты (без учёта субъективных оценок очных собеседований). 21.10.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="32" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>№</t>
@@ -559,7 +552,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Критерий оценки</t>
+          <t>Критерий оценки анкеты</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -569,12 +562,13 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Отрицательные сигналы (−)</t>
+          <t>Отрицательные сигналы (−)
+[Риски анкеты]</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Допустимое использование в ИИ / алгоритме</t>
+          <t>Логика первичной обработки ИИ</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -584,7 +578,7 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Уточняющие вопросы при неопределённости</t>
+          <t>Контекстные уточнения в диалоге анкеты</t>
         </is>
       </c>
     </row>
@@ -595,45 +589,44 @@
       <c r="B5" s="5" t="inlineStr">
         <is>
           <t>Мотивация и осознанность выбора
-(+ Сфера интересов и Источник прихода)</t>
+(Источник и цели)</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>• Чёткие личные и профессиональные цели
-• Осознанный источник прихода: личный поиск на сайте ГИМ, рекомендации действующих волонтёров, интерес к выставкам
-• Партнёрская мотивация («хочу помочь музею», «применить навыки для посетителей»)
-• Совпадение научных интересов с профилем ГИМ (археология, история России, архивы, музеология)
-• Фокус на 1–2 профильных направлениях</t>
+          <t>• Личная инициатива (поиск через сайт ГИМ, интерес к выставкам, рекомендации волонтёров)
+• Партнёрская мотивация: кандидат пишет, чем хочет быть полезен музею и посетителям
+• Совпадение интересов с историей, культурой и профилем ГИМ
+• Осознанный фокус на 1–2 направлениях</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>• Административное принуждение от вуза («преподаватель сказал», «заставили в чате группы ради зачёта по практике») — главный триггер оценки 0 в 2025 г.!
-• Потребительская мотивация в 1–2 слова («Опыт», «Практика», «Интересно»)
-• Жёсткая фиксация исключительно на фондах («хочу только в фонд» — риск «мёртвой души»)
-• «Ковровый выбор» всех направлений подряд (все 5 галочек) без понимания их различий</t>
+          <t>• Административное принуждение от вуза («сказали в чате группы», «от преподавателя для зачёта по практике»)
+• Потребительская мотивация («просто опыт», «бесплатный вход»)
+• Скрытый поиск работы («с перспективой трудоустройства в музей»)
+• «Ковровый выбор» всех направлений подряд (4–5 галочек) без понимания специфики</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>• Оценка глубины мотивации и искренности интереса
-• Фильтрация административно направленных студентов от мотивированных добровольцев
-• ❌ ЗАПРЕТ: не отказывать автоматически за лаконичность, если есть профильный интерес</t>
+          <t>• Фильтрация анкет «для галочки» от реальных добровольцев
+• Детекция риска «скрытого трудоустройства» (волонтёрство ≠ стажировка с наймом)
+• Запрос конкретизации при выборе &gt;2 направлений</t>
         </is>
       </c>
       <c r="F5" s="6" t="inlineStr">
         <is>
           <t>«Мотивация: высокая / средняя / формальная (риск принудительной практики)»
-Цитата-обоснование.
-Совпадение научных интересов с профилем музея: да / нет.</t>
+Маркер: «Скрытый поиск работы: да / нет»
+Цитата-обоснование из анкеты.</t>
         </is>
       </c>
       <c r="G5" s="6" t="inlineStr">
         <is>
-          <t>• Если источник «ВУЗ/преподаватель»: «Что именно побудило вас подать заявку: личный интерес к истории или необходимость закрыть практику?»
-• Если выбраны все направления подряд: «Какое одно направление для вас действительно в приоритете и почему?»
-• Если ответ краткий: «Что конкретно в экспозиции ГИМ вам ближе всего?»</t>
+          <t>• Если источник вуз: «Что именно привлекает вас в ГИМ помимо закрытия учебного плана?»
+• Если выбраны все направления: «Какое одно направление для вас ключевое и почему?»
+• Если указан поиск работы: «Программа волонтёрская. Рассматриваете ли вы участие без гарантии найма?»</t>
         </is>
       </c>
     </row>
@@ -643,44 +636,43 @@
       </c>
       <c r="B6" s="8" t="inlineStr">
         <is>
-          <t>Опыт и навыки
-(+ Софт-скиллы и «Суперсила»)</t>
+          <t>Опыт и прикладные навыки
+(Компетенции и суперсила)</t>
         </is>
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>• Профильный опыт (музеи, выставки, архивы, археологические экспедиции, инклюзия)
-• Прикладные навыки: фото, видео, монтаж, дизайн, тексты, иностранные языки B1+
-• Опыт школьных/студенческих олимпиад («Музеи. Парки. Усадьбы», Всерос)
-• Осознанная «Суперсила» с привязкой к делу и самоиронией (усидчивость с документами, стрессоустойчивость, умение просто объяснять сложное)</t>
+          <t>• Профильный опыт (музеи, выставки, архивы, экспедиции, инклюзивные проекты)
+• Прикладные навыки: фото, видео, монтаж, дизайн, тексты, языки B1+, ведение групп
+• Осознанная «Суперсила»: конкретные прикладные софт-скиллы (усидчивость, стрессоустойчивость, умение просто объяснять сложное)</t>
         </is>
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
-          <t>• Пустые графы в опыте без попытки описать смежные навыки
-• Формализм в «Суперсиле»: прочерк, «не знаю», штампы («всегда встаю по утрам», «коммуникабельность» в 1 слово), пафосные цитаты без связи с задачами
-• Не указано, чем именно кандидат может быть полезен музею</t>
+          <t>• Пустые графы опыта при отсутствии описания любых полезных навыков
+• Формализм в графе суперсилы (прочерк, «не знаю», пустые штампы)
+• Претензия исключительно на академическую работу при отказе от помощи на событиях музея</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
         <is>
-          <t>• Мэтчинг компетенций под направления музея
-• Анализ адекватности самооценки и софт-скиллов по ответу о суперсиле
-• ❌ ЗАПРЕТ: не отсекать кандидатов с непрофильным образованием (инженеры, медики) при наличии мотивации</t>
+          <t>• Мэтчинг подтверждённых компетенций с 5 направлениями музея
+• Анализ софт-скиллов по развёрнутости ответа о суперсиле
+• ❌ Не отсекать кандидатов с непрофильным образованием (инженеры, медики) при наличии мотивации</t>
         </is>
       </c>
       <c r="F6" s="9" t="inlineStr">
         <is>
           <t>«Подтверждённые hard skills: [список]»
 «Качество софт-скиллов (по суперсиле): зрелое / формальное»
-«Рекомендованные направления ГИМ».</t>
+«Рекомендованный трек волонтёрства».</t>
         </is>
       </c>
       <c r="G6" s="9" t="inlineStr">
         <is>
-          <t>• По суперсиле: «Приведите пример, когда ваша суперсила помогла решить сложную или нестандартную задачу?»
-• Для медиа/проектов: «Есть ли готовые примеры ваших текстов, фото, видео или сценариев мероприятий?»
-• «В чём именно вам хотелось бы попрактиковаться в ГИМ?»</t>
+          <t>• По суперсиле: «Приведите пример ситуации, где ваша суперсила помогла решить задачу?»
+• Для медиа/дизайна: «Есть ли готовые ссылки на ваши фото, видео или тексты?»
+• «В чём именно хотелось бы попрактиковаться в ГИМ?»</t>
         </is>
       </c>
     </row>
@@ -691,40 +683,44 @@
       <c r="B7" s="5" t="inlineStr">
         <is>
           <t>Курс обучения и нагрузка
-(+ Конфликт параллельных проектов)</t>
+(ФАКТОР ВЫСОКОГО РИСКА НА СКРИНИНГЕ)</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>• Старшие курсы (2–4 курс бакалавриата, магистратура), выпускники со стабильным графиком
-• Наличие свободного времени в графике (выходные, будни вечер)
-• Реалистичное понимание объёма времени (от 16 часов в месяц)</t>
+          <t>• Оконченное образование (выпускники) / стабильная работа с предсказуемым графиком
+• Заочная, вечерняя форма обучения или свободный график
+• Старшие выпускные курсы с минимальной аудиторной нагрузкой
+• Наличие свободных часов в выходные и вечерами (от 16 ч/мес)</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>• 1-й курс бакалавриата (статистический риск выгорания и завала первой сессии)
-• ⚠️ УЧАСТИЕ В ДРУГИХ СХОЖИХ ПРОЕКТАХ ПРЯМО СЕЙЧАС (волонтёрство в Третьяковке/Пушкинском, работа в другом музее, актив в студсовете одновременно) — риск распыления и нулевой выработки часов!
-• Высокая загруженность (очная учёба + full-time работа без гибкого графика)</t>
+          <t>• ⚠️ ОЧНОЕ ОБУЧЕНИЕ В ВУЗЕ / СПО (БОЛЬШОЙ МИНУС НА ЭТАПЕ АНКЕТЫ):
+  1) Пары с 9:00 до 16:00-18:00 блокируют будни -&gt; КРИТИЧЕСКИЙ КОНФЛИКТ С ФОНДАМИ (фонды работают 10-18 по будням!)
+  2) Сессионные провалы 2 раза в год (зима/лето) в пик музейных событий
+  3) 1-й курс очного бакалавриата - максимальный риск перегрузки
+• ⚠️ ПАРАЛЛЕЛЬНОЕ УЧАСТИЕ В ДРУГИХ ПРОЕКТАХ ПРЯМО СЕЙЧАС (музеи, студсовет) - мультизанятость и риск нулевой выработки часов</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>• Индикация рисков доступности и конфликта расписаний
-• Подсвечивание маркера «Параллельные проекты / Мультизанятость»
-• ❌ СТРОГИЙ ЗАПРЕТ: не ставить автоматический отказ первокурсникам и занятым людям, а выносить вопрос о часах на интервью</t>
+          <t>• АВТОМАТИЧЕСКИЙ ШТРАФ В БЛОКЕ НАГРУЗКИ ЗА ОЧНОЕ ОБУЧЕНИЕ
+• БЛОКИРУЮЩИЙ АЛЕРТ: если очник выбрал ТОЛЬКО фонды, система СРАЗУ выдаёт предупреждение и требует сменить трек или подтвердить свободное посещение
+• Проверка готовности очников выходить строго в выходные дни</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>«Маркер нагрузки: 1 курс / совмещение с работой / параллельные проекты [указать какие]»
-Рекомендация: детально согласовать график дежурств и приоритет ГИМ на очном интервью.</t>
+          <t>«⚠️ Статус: Студент очного отделения (риск блокировки будней и сессий)»
+«Конфликт с фондовым графиком: КРИТИЧЕСКИЙ / НЕТ»
+«Параллельные проекты: [список]».</t>
         </is>
       </c>
       <c r="G7" s="6" t="inlineStr">
         <is>
-          <t>• По параллельным проектам: «Вы указали участие в проекте [X]. Сколько конкретно часов в неделю вы сможете гарантированно уделять ГИМ без ущерба для текущих обязательств?»
-• «Какой график вам удобнее: регулярные дежурства по субботам/воскресеньям или разовые акции?»</t>
+          <t>• Очнику при выборе фондов: «Фондовая работа идёт ТОЛЬКО по будням с 10:00 до 18:00. При очном обучении это невозможно без свободного посещения. Сможете ли вы присутствовать в эти часы или переключимся на выходные дни?»
+• «Участвуете ли вы прямо сейчас в других проектах? Сколько часов в неделю свободно для ГИМ?»</t>
         </is>
       </c>
     </row>
@@ -734,40 +730,40 @@
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>Цифровой след и полнота анкеты</t>
+          <t>Цифровой след и полнота анкеты
+(Качество данных и связь)</t>
         </is>
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
           <t>• Развёрнутая, структурированная анкета с законченными мыслями
-• Корректная работающая ссылка на страницу ВКонтакте для оперативной связи
-• Открытый диалог при заполнении</t>
+• Корректная работающая ссылка на профиль ВКонтакте (основной рабочий канал музея)</t>
         </is>
       </c>
       <c r="D8" s="9" t="inlineStr">
         <is>
-          <t>• Полупустая анкета («телеграфный стиль», ответы по 1–2 слова)
+          <t>• Полупустая анкета («телеграфный стиль», отписки по 1–2 слова)
 • Не указана ссылка на ВК (указан только телефон)
-• Закрытый профиль ВК / пустая страница без активности</t>
+• Закрытый профиль ВК без возможности написать личное сообщение</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
         <is>
-          <t>• Проверка полноты заполнения полей
-• Верификация канала связи (ВК — основной рабочий инструмент музея)
-• ❌ ЗАПРЕТ: не парсить закрытые страницы и не снижать оценку за настройки приватности</t>
+          <t>• Проверка полноты заполнения смысловых полей
+• Автоматическая валидация синтаксиса и доступности ссылки ВК
+• ❌ Не парсить приватные данные и не оценивать личные фото/посты</t>
         </is>
       </c>
       <c r="F8" s="9" t="inlineStr">
         <is>
-          <t>«Полнота анкеты: высокая / средняя / низкая (телеграфный стиль)»
-«Статус канала связи: VK предоставлен / требуется подтвердить контакт».</t>
+          <t>«Полнота анкеты: высокая / средняя / низкая»
+«Канал связи VK: подтверждён / требует уточнения».</t>
         </is>
       </c>
       <c r="G8" s="9" t="inlineStr">
         <is>
-          <t>• «Координация смен волонтёров проходит в беседах ВКонтакте. Будет ли у вас возможность оперативно быть на связи?»
-• «Готовы ли вы открыть личные сообщения для куратора?»</t>
+          <t>• «Координация волонтёров проходит в беседах ВКонтакте. Будет ли у вас возможность оперативно быть на связи?»
+• «Готовы ли вы открыть личные сообщения для куратора программы?»</t>
         </is>
       </c>
     </row>
@@ -778,40 +774,38 @@
       <c r="B9" s="5" t="inlineStr">
         <is>
           <t>Логистика и бытовые вопросы
-(+ График музейных событий)</t>
+(География и график)</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
           <t>• Проживание в Москве или ближнем Подмосковье
 • Реалистичная оценка времени на дорогу до Красной площади
-• Готовность к очным сменам в дни проведения музейных мероприятий</t>
+• Готовность к очным сменам в дни мероприятий музея (выходные, вечера четверга/пятницы)</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>• Проживание в других регионах России (при выборе очных направлений)
-• Несовместимость графика с днями ключевых акций музея (четверги/пятницы вечер, выходные дни)</t>
+          <t>• Проживание в удалённых городах РФ при выборе очных треков
+• Несовместимость графика с днями ключевых музейных событий</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>• Проверка территориальной доступности для очных смен
-• Маршрутизация иногородних на удалённые треки (медиа, тексты, дизайн)
-• ❌ ЗАПРЕТ: не отсекать иногородних студентов московских вузов</t>
+          <t>• Гео-проверка: автоматическая маршрутизация иногородних кандидатов на дистанционный трек (медиа, тексты, дизайн)
+• ❌ Не отсекать иногородних студентов московских вузов, живущих в общежитиях</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
           <t>«Локация: Москва / Иногородний»
-«Формат участия: очный / возможен онлайн (медиа)»
-«Готовность к сменам в выходные дни».</t>
+«Формат участия: очный / рекомендован дистанционный (медиа)».</t>
         </is>
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>• «Планируете ли вы очное участие в Москве или рассматриваете дистанционные задачи (медиа, переводы, тексты)?»
-• «Удобно ли вам участвовать в мероприятиях по выходным и в вечернее время?»</t>
+          <t>• Иногородним: «Вы указали город вне Москвы. Рассматриваете ли вы дистанционные задачи (медиа, дизайн) или готовы приезжать очно?»
+• «Удобно ли вам участвовать в мероприятиях в выходные дни?»</t>
         </is>
       </c>
     </row>
@@ -826,32 +820,32 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
-    <col width="32" customWidth="1" min="6" max="6"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Детерминированные правила (Hard Rules — вне шкалы ИИ)</t>
+          <t>Детерминированные фильтры первичного скрининга (Hard Rules)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Правила проверяются строго кодом по принципу Да/Нет, модель ИИ не принимает субъективных решений</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="26" customHeight="1">
+          <t>Проверяются программным кодом строго по правилам Да/Нет до передачи анкеты на оценку нейросетью</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="28" customHeight="1">
       <c r="A4" s="10" t="inlineStr">
         <is>
           <t>№</t>
@@ -859,7 +853,7 @@
       </c>
       <c r="B4" s="10" t="inlineStr">
         <is>
-          <t>Правило</t>
+          <t>Правило фильтрации</t>
         </is>
       </c>
       <c r="C4" s="10" t="inlineStr">
@@ -869,12 +863,12 @@
       </c>
       <c r="D4" s="10" t="inlineStr">
         <is>
-          <t>Источник данных в анкете</t>
+          <t>Источник в анкете</t>
         </is>
       </c>
       <c r="E4" s="10" t="inlineStr">
         <is>
-          <t>Логика работы системы</t>
+          <t>Логика работы скрининга</t>
         </is>
       </c>
       <c r="F4" s="10" t="inlineStr">
@@ -883,18 +877,18 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="65" customHeight="1">
+    <row r="5" ht="70" customHeight="1">
       <c r="A5" s="4" t="n">
         <v>1</v>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Возраст 18+</t>
+          <t>Возрастной ценз 18+</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>Детерминированное правило (18+ обязателен)</t>
+          <t>Детерминированный отсев (Hard Rule)</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
@@ -904,72 +898,102 @@
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>Если возраст &lt; 18 лет: заявка блокируется для очного интервью, выставляется статус eligibility.age_over_18 = False. Решение не отдаётся на усмотрение ИИ.</t>
+          <t>Если возраст &lt; 18 лет: анкета блокируется для очного отбора (статус eligibility.age_over_18 = false). Программа закрытого типа 18+.</t>
         </is>
       </c>
       <c r="F5" s="6" t="inlineStr">
         <is>
-          <t>Красный бейдж: «Несовершеннолетний (18-)». Причина: правила закрытой волонтёрской программы музея.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="65" customHeight="1">
+          <t>Красный бейдж: «Несовершеннолетний (18-)».</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="70" customHeight="1">
       <c r="A6" s="7" t="n">
         <v>2</v>
       </c>
       <c r="B6" s="8" t="inlineStr">
         <is>
-          <t>Согласие на обработку данных (ОПД)</t>
+          <t>Согласие на ОПД</t>
         </is>
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>Обязательное условие отправки</t>
+          <t>Блокирующая валидация формы</t>
         </is>
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
-          <t>Чекбокс согласия со ссылкой на политику ГИМ (shm.ru)</t>
+          <t>Чекбокс согласия со ссылкой на политику shm.ru</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
         <is>
-          <t>Валидация на клиенте и backend. Без активного согласия отправка анкеты физически блокируется.</t>
+          <t>Без активного согласия форма физически не отправляется на сервер.</t>
         </is>
       </c>
       <c r="F6" s="9" t="inlineStr">
         <is>
-          <t>Зелёный бейдж: «Согласие на ОПД получено».</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="65" customHeight="1">
+          <t>Зелёный бейдж: «Согласие ОПД получено».</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="70" customHeight="1">
       <c r="A7" s="4" t="n">
         <v>3</v>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Наличие канала связи</t>
+          <t>Конфликт «Очник + Фонды»</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>Валидация контактных данных</t>
+          <t>Логический конфликт расписания (Hard Alert)</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
+          <t>Статус «Студент очно» + выбор направления «Фондовая работа»</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>Если кандидат учится очно и выбрал ТОЛЬКО фонды: форма выдаёт диалоговое предупреждение о несовместимости графика будней (10:00–18:00). Если кандидат не подтверждает свободный график — анкета не рекомендуется к собеседованию.</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>Оранжевый бейдж: «Конфликт расписания: очник претендует на фонды».</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="70" customHeight="1">
+      <c r="A8" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>Валидация канала связи</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>Проверка контактных данных</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
           <t>Поле «Ссылка на страницу ВК» + Email</t>
         </is>
       </c>
-      <c r="E7" s="6" t="inlineStr">
-        <is>
-          <t>Проверка синтаксиса ссылки/профиля ВК. Если ссылка некорректна, система просит исправить её до финализации анкеты.</t>
-        </is>
-      </c>
-      <c r="F7" s="6" t="inlineStr">
-        <is>
-          <t>Статус контакта: «VK верифицирован» / «Требуется ручное уточнение контакта».</t>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>Проверка формата ссылки. Если указан только номер телефона или битая ссылка, форма просит ввести корректный профиль ВК для связи.</t>
+        </is>
+      </c>
+      <c r="F8" s="9" t="inlineStr">
+        <is>
+          <t>Статус: «VK верифицирован» / «Требуется ручное уточнение».</t>
         </is>
       </c>
     </row>
@@ -988,27 +1012,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="35" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="35" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
     <col width="38" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Специфика 5 направлений волонтёрской деятельности ГИМ</t>
+          <t>Специфика направлений ГИМ: требования к графику и совместимость</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Используется для маршрутизации кандидата и формулирования целевых вопросов для интервью</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="26" customHeight="1">
+          <t>Используется для первичной проверки совместимости графика кандидата с выбранным направлением</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="28" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Направление</t>
@@ -1016,26 +1040,26 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Суть деятельности</t>
+          <t>График и режим работы</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Профильные навыки</t>
+          <t>Совместимость с очным обучением</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Типичный риск / Специфика</t>
+          <t>Профильные компетенции</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Вопрос для диалога / интервью</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="70" customHeight="1">
+          <t>Вопрос при заполнении анкеты</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="75" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
           <t>Фондовое направление</t>
@@ -1043,26 +1067,26 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>Помощь хранителям в фондах музея, работа с документами, каталогизация, учёт предметов.</t>
+          <t>СТРОГО БУДНИ с 10:00 до 17:00–18:00 (хранилища закрыты по выходным)</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>Архивное дело, история, аккуратность, усидчивость, знание спецдисциплин.</t>
+          <t>❌ КРАЙНЕ НИЗКАЯ. Очные студенты физически на парах в эти часы. Доступно только выпускникам, вечерникам или при официальном свободном посещении.</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>Слишком высокий конкурс, мест физически мало. Риск «мёртвой души», если кандидат согласен только на фонд.</t>
+          <t>Архивное дело, история, усидчивость, аккуратность, работа с описями.</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>«Какие конкретно коллекции или фонды вас привлекают? Рассматриваете ли участие в других направлениях ГИМ?»</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="70" customHeight="1">
+          <t>«Фонды работают только по будням с 10 до 18. Сможете ли вы присутствовать в эти часы без ущерба для учёбы?»</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="75" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
         <is>
           <t>Проектное направление</t>
@@ -1070,26 +1094,26 @@
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>Разработка и проведение квестов, мастер-классов, викторин, образовательных игр для гостей.</t>
+          <t>Выходные дни, каникулы, праздничные даты, вечерние часы</t>
         </is>
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>Креативность, сценарии, работа с детьми/семьями, ораторские навыки, педагогика.</t>
+          <t>✅ ВЫСОКАЯ. Идеально подходит очным студентам: разработка квестов и проведение мастер-классов проходит по субботам и воскресеньям.</t>
         </is>
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
-          <t>Требуется готовность доводить идею до финала и согласовывать с методистами музея.</t>
+          <t>Креативность, сценарии, работа с детьми/семьями, педагогика.</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
         <is>
-          <t>«Какие форматы мероприятий вам ближе: разработка сценария квеста, проведение мастер-класса или экскурсия-игра?»</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="70" customHeight="1">
+          <t>«Какие форматы вам ближе: проведение квестов, мастер-классов или разработка образовательных игр?»</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="75" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
           <t>Организационное направление</t>
@@ -1097,26 +1121,26 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>Помощь в логистике, навигация потоков посетителей на масштабных событиях, стойки информации.</t>
+          <t>Выходные дни, дни выставочных открытий, четверги/пятницы вечер</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>Стрессоустойчивость, коммуникабельность, энергичность, ориентация в здании музея.</t>
+          <t>✅ ВЫСОКАЯ. Основная нагрузка приходится на дни акций («Ночь музеев», фестивали, выставки) по выходным.</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>Пиковые физические нагрузки в дни акций («Ночь музеев», фестивали, выставки).</t>
+          <t>Коммуникабельность, навигация, стрессоустойчивость, ориентация в музее.</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>«С какой категорией посетителей вам комфортнее работать: дети, молодёжь, взрослые или пожилые гости?»</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="70" customHeight="1">
+          <t>«С какой категорией посетителей вам комфортнее работать: дети, молодёжь или взрослые гости?»</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="75" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
         <is>
           <t>Инклюзивное направление</t>
@@ -1124,26 +1148,26 @@
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>Адаптация музейных программ для людей с ОВЗ, тактильные экскурсии, сопровождение.</t>
+          <t>По расписанию инклюзивных мероприятий (будни вечер / выходные)</t>
         </is>
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>Эмпатия, логопедия, дефектология, жестовый язык, опыт работы с людьми с инвалидностью.</t>
+          <t>⚖️ СРЕДНЯЯ. Зависит от расписания конкретных программ адаптации.</t>
         </is>
       </c>
       <c r="D8" s="9" t="inlineStr">
         <is>
-          <t>Требуется деликатность, ответственность и психологическая устойчивость.</t>
+          <t>Эмпатия, дефектология, сурдокоммуникация, опыт работы с людьми с ОВЗ.</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
         <is>
-          <t>«Был ли у вас опыт общения или волонтёрства с людьми с особыми потребностями? Готовы пройти спецподготовку?»</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="70" customHeight="1">
+          <t>«Был ли у вас опыт общения или волонтёрства с людьми с особыми потребностями?»</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="75" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
           <t>Медиа волонтёрство</t>
@@ -1151,26 +1175,26 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Фото- и видеосъёмка, подготовка постов, контент-планов, репортажей, монтаж рилсов, дизайн афиш.</t>
+          <t>Гибкий / удалённый график (с выездом на съёмки по согласованию)</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>SMM, копирайтинг, графический дизайн, видеомонтаж, фотосъёмка, знание трендов.</t>
+          <t>✅ МАКСИМАЛЬНАЯ. Монтаж, тексты, дизайн и SMM можно выполнять дистанционно в удобное время.</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>Возможна удалённая работа, но критичны дедлайны и соблюдение визуального брендбука музея.</t>
+          <t>SMM, дизайн, видеомонтаж, фотосъёмка, копирайтинг.</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>«Что вам ближе: съёмка репортажей, видеомонтаж, написание текстов или дизайн? Пришлите примеры ваших работ»</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="70" customHeight="1">
+          <t>«Что вам ближе: видео, фото, тексты или дизайн? Прикрепите ссылки на примеры ваших работ»</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="75" customHeight="1">
       <c r="A10" s="8" t="inlineStr">
         <is>
           <t>Пока не определился</t>
@@ -1178,22 +1202,22 @@
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>Кандидат хочет помогать музею, но пока не знает внутренних процессов и возможностей.</t>
+          <t>Определяется после скрининга доступности</t>
         </is>
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>Открытость новому опыту, широкий кругозор, готовность учиться.</t>
+          <t>⚖️ Маршрутизируется системой исходя из графика занятости кандидата.</t>
         </is>
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
-          <t>Нужна профориентация на этапе анкеты, чтобы предложить подходящий стартовый трек.</t>
+          <t>Широкий кругозор, открытость новому, готовность помогать.</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
         <is>
-          <t>«Что вам ближе в свободное время: общение с людьми, творческая работа за компьютером или исследовательский труд?»</t>
+          <t>«Сколько часов в месяц вы готовы уделять и в какие дни (будни или выходные)?»</t>
         </is>
       </c>
     </row>
@@ -1212,163 +1236,167 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="35" customWidth="1" min="2" max="2"/>
     <col width="38" customWidth="1" min="3" max="3"/>
-    <col width="36" customWidth="1" min="4" max="4"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Аналитический срез реальных анкет 2024–2025 гг. и решений кураторов ГИМ</t>
+          <t>Системные правила первичной оценки входных анкет (Stage 1 Screening)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="11" t="inlineStr">
-        <is>
-          <t>Базируется на выборке из 180+ анкет (materials/gim): выявление ключевых драйверов высоких и низких оценок</t>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Без учёта субъективных оценок очных собеседований (с учётом 20% погрешности кураторских оценок)</t>
         </is>
       </c>
     </row>
     <row r="4" ht="28" customHeight="1">
-      <c r="A4" s="12" t="inlineStr">
-        <is>
-          <t>Категория анализа</t>
-        </is>
-      </c>
-      <c r="B4" s="12" t="inlineStr">
-        <is>
-          <t>Фактический паттерн из данных</t>
-        </is>
-      </c>
-      <c r="C4" s="12" t="inlineStr">
-        <is>
-          <t>Статистика / Примеры из таблиц</t>
-        </is>
-      </c>
-      <c r="D4" s="12" t="inlineStr">
-        <is>
-          <t>Вывод и рекомендация для нашего ИИ</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="110" customHeight="1">
+      <c r="A4" s="11" t="inlineStr">
+        <is>
+          <t>Фактор скрининга</t>
+        </is>
+      </c>
+      <c r="B4" s="11" t="inlineStr">
+        <is>
+          <t>Признак в анкете кандидата</t>
+        </is>
+      </c>
+      <c r="C4" s="11" t="inlineStr">
+        <is>
+          <t>Риск для музея / Обоснование</t>
+        </is>
+      </c>
+      <c r="D4" s="11" t="inlineStr">
+        <is>
+          <t>Алгоритмическое действие системы</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="95" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>1. Феномен оценки 0
-(Отказ без собеседования)</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>ВЕСНА 2025: 27 анкет получили 0 баллов из-за административного принуждения со стороны вуза (ГУП / МГОУ). Кандидатов обязали подать заявку ради учебной практики.</t>
+          <t>1. Очное обучение в вузе
+(Большой системный минус)</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>Статус: «Студент (очно)»
+Курс: 1–4 курс бакалавриата / специалитета</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>Источник: «Сказали в чате группы», «Преподаватель», «Администрация вуза».
-Ожидания: «Опыт», «Пройти практику».
-Суперсила: «-», «Не знаю», «Всегда встаю по будильнику».</t>
+          <t>Блокировка дневного времени по будням (9:00–18:00). Сессионные провалы дважды в год (декабрь-январь и май-июнь) — выпадение волонтёра в самые пиковые музейные дни. Риск завала учёбы.</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>ИИ должен выявлять отсутствие личной мотивации и шаблонные отписки «для галочки». Задавать проверочный вопрос о личной цели участия.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="110" customHeight="1">
+          <t>• Штраф в блоке нагрузки (-1.0 балл).
+• Автоматическая блокировка направления «Фонды» без подтверждения свободного графика.
+• Обязательная проверка готовности к сменам в выходные.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="95" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>2. Параллельные проекты
-(Риск мультизанятости)</t>
-        </is>
-      </c>
-      <c r="B6" s="8" t="inlineStr">
-        <is>
-          <t>Кандидаты, которые прямо сейчас волонтёрят в 2–3 музеях (Пушкинский, Третьяковка, Музей Москвы) или работают full-time, в 2024 г. показали выработку часов &lt; 10 ч/год или выбыли.</t>
+          <t>2. Мультизанятость прямо сейчас
+(Параллельные проекты)</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>В графе опыта указано текущее активное волонтёрство в 2+ других музеях/организациях либо full-time работа + учёба</t>
         </is>
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>Примеры: волонтёр НИУ ВШЭ + Пушкинский + Третьяковка (активность 23 ч); работа в РГАЛИ + Artlife (активность снижена).
-У кандидата с 3 проектами активность = 0 ч.</t>
+          <t>Распыление внимания, накладка смен, приоритет другому проекту при аврале. Высокий риск нулевой выработки часов.</t>
         </is>
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
-          <t>Не отказывать автоматически, но маркировать как риск нехватки времени. ИИ генерирует вопрос о распределении часов между проектами.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="110" customHeight="1">
+          <t>• Маркировка флагом «Параллельные проекты».
+• Формирование проверочного вопроса о гарантированных часах именно для ГИМ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="95" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>3. Портрет «Звёздного волонтёра»
-(Активность &gt; 30–300 часов)</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>Студенты 2–4 курсов (РГГУ, МГУ, ВШЭ, МПГУ) или выпускники с профильным интересом к истории/музеологии, имеющие опыт олимпиад («Музеи. Парки. Усадьбы») или практики.</t>
+          <t>3. Административное принуждение
+(Формальная практика)</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>Источник: «Преподаватель», «Администрация вуза», «Сказали в чате группы ради зачёта».
+Ожидания: «Опыт» в одно слово, «Пройти практику».</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>Рекордсмен 2024 г. (317 часов!): РГГУ, 3 курс, олимпиада «Музеи. Парки. Усадьбы», чёткое понимание специфики квестов и фондов, суперсила — стрессоустойчивость.</t>
+          <t>Нулевая внутренняя мотивация. Человек пришёл ради галочки/зачёта, уйдёт сразу после подписания дневника практики.</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>ИИ должен начислять повышенный скоринг за профильные олимпиады, конкретный фокус в направлениях и зрелую рефлексию.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="110" customHeight="1">
+          <t>• Маркировка как «Формальная заявка».
+• Запрос развёрнутого ответа о личном интересе к музею до передачи координатору.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="95" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>4. Графа «Суперсила» как фильтр
-софт-скиллов</t>
-        </is>
-      </c>
-      <c r="B8" s="8" t="inlineStr">
-        <is>
-          <t>Кураторы используют ответ о суперсиле как маркер зрелости и чувства юмора. Успешные кандидаты пишут о прикладных софт-скиллах, отсеянные — ставят прочерк или банальность.</t>
+          <t>4. Скрытый поиск работы
+(Headhunting trap)</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>Ожидания: «С перспективой трудоустройства в штат», «Смена работы», «Поиск вакансий в музее».</t>
         </is>
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>Балл 3: «Въедливость, могу долго сидеть над монотонной задачей», «Умею говорить забавным голосом и объяснять сложное просто».
-Балл 0: «-», «Коммуникабельность», «Вставать по утрам».</t>
+          <t>Волонтёрская программа закрытого типа не является агентством по найму. Соискатель уходит, как только понимает, что вакансию не предложат, или находит платную работу.</t>
         </is>
       </c>
       <c r="D8" s="9" t="inlineStr">
         <is>
-          <t>ИИ анализирует текстовое качество ответа на вопрос о суперсиле: содержательность, самоирония, прикладной характер для работы с людьми/экспонатами.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="110" customHeight="1">
+          <t>• Маркировка флагом «Скрытый поиск работы».
+• Модель разъясняет кандидату волонтёрский статус программы прямо в диалоге.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="95" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>5. «Ковровый выбор» направлений</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>Кандидаты с баллом 0 и 1 почти всегда отмечают ВСЕ доступные направления подряд (Организация, Проекты, Фонды, Инклюзия).</t>
+          <t>5. «Ковровый выбор» направлений
+(Отсутствие фокуса)</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>Выбраны все доступные направления одновременно (Орг + Проекты + Фонды + Инклюзия + Медиа) без профильного опыта.</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>В анкетах со Score 0: 4–5 направлений выбраны одновременно без единого комментария в опыте.
-В анкетах со Score 3: выбрано 1–2 сфокусированных трека.</t>
+          <t>Кандидат не понимает различий между задачами, заполняет анкету на автомате.</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>ИИ детектирует выбор &gt;3 направлений как маркер неопределённости и формирует диалоговое уточнение: «Какое направление для вас ключевое?»</t>
+          <t>• Детекция выбора &gt;2 разнородных направлений.
+• Диалоговый вопрос бота: «Какое одно направление для вас ключевое?»</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: add synthetic candidates for testing and update selection criteria
</commit_message>
<xml_diff>
--- a/docs/Критерии_отбора_ГИМ.xlsx
+++ b/docs/Критерии_отбора_ГИМ.xlsx
@@ -8,10 +8,11 @@
   </bookViews>
   <sheets>
     <sheet name="5 Критериев отбора" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Шкала оценок кураторов 0-3" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Направления ГИМ" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Формат выгрузки для куратора" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Объективные фильтры" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="4 Контрастных сценария" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Шкала оценок кураторов 0-3" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Направления ГИМ" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Формат выгрузки для куратора" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Объективные фильтры" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -57,6 +58,41 @@
       <name val="Calibri"/>
       <color rgb="00000000"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00333333"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00C00000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00375623"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00C00000"/>
+      <sz val="12"/>
     </font>
   </fonts>
   <fills count="7">
@@ -123,7 +159,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -159,6 +195,23 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -547,7 +600,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Сверено с официальным ТЗ («Анкета волонтёра») и ответами заказчика от 21.10.2026 (docs/06-gim-stakeholder-answers.md)</t>
+          <t>Сверено с ТЗ и ответами ГИМ (21.10.2026). 4 эталонных тестовых сценария: см. лист «4 Контрастных сценария»</t>
         </is>
       </c>
     </row>
@@ -836,6 +889,408 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="52" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="36" customWidth="1" min="9" max="9"/>
+    <col width="30" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Государственный исторический музей (ГИМ) · 4 Контрастных сценария: распределение оценок [0, 2, 3, ТРЕБУЕТ ПРОВЕРКИ]</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Полные ответы на ВСЕ 19 вопросов анкеты ГИМ. Чёткое распределение: один с 0, один с 2, один с 3 и один со статусом ТРЕБУЕТ ПРОВЕРКИ. 21.10.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="28" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Тип сценария</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Кандидат и статус</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>ПОЛНЫЕ ВХОДНЫЕ ОТВЕТЫ НА ВСЕ 19 ВОПРОСОВ АНКЕТЫ ГИМ</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Ожидаемое направление</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Кураторский балл</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Сильные стороны</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Возможные проблемы (Риски)</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Ожидаемые вопросы для интервью</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>Что проверяет кейс</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="290" customHeight="1">
+      <c r="A5" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Мотивированный первокурсник
+(Исключение по нагрузке)</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Алексей Смирнов, 18 лет
+Студент (очно), 1 курс
+НИУ ВШЭ (История)</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>1. Согласие на ОПД: Да, даю согласие
+2. ФИО: Смирнов Алексей Дмитриевич
+3. Электронная почта: smirnov.alex.hse@gmail.com
+4. Ссылка на страницу ВК: https://vk.com/smirnov_alex_hse
+5. Дата рождения: 15.09.2008 (18 лет)
+6. Ваш нынешний статус: Студент
+7. ВУЗ: Национальный исследовательский университет «Высшая школа экономики» (НИУ ВШЭ)
+8. ВУЗ (Другое): —
+9. Факультет: Факультет гуманитарных наук, ОП «История»
+10. Курс: 1 курс бакалавриата
+11. Сфера научных интересов: История России XVII века, Смутное время, формирование сословий
+12. Опыт работы, стажировки, проекты: Волонтёр школьных исторических чтений, проведение Дня открытых дверей в лицее ВШЭ (навигация гостей, регистрация участников)
+13. Иностранные языки (B1 и выше): Английский язык (B2)
+14. Почему Вы выбрали волонтёрскую программу Исторического музея?: С детства посещаю ГИМ. Для меня ГИМ — это главный музей страны по профилю моего исторического образования. Хочу быть полезным музею и развиваться в музейной среде.
+15. Чего Вы ожидаете от волонтёрства в Историческом музее?: Применить академические знания на практике, научиться работать с аудиторией, участвовать в проведении квестов и интерактивов для подростков.
+16. Сколько времени Вы готовы уделять добровольческой деятельности в месяц?: 32 часа в месяц (обучаюсь по индивидуальному плану: вторник и четверг без пар, все выходные свободны. Других проектов нет).
+17. Ваши хобби: Настольные исторические стратегии, чтение архивных мемуаров, походы в музеи
+18. В работу какого направления Вы бы хотели включиться?: Проектное направление (разработка квестов/мастер-классов для культурно-массовых мероприятий)
+19. Откуда Вы узнали о Волонтерской программе?: Сайт Исторического музея</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>Проектное направление
+(квесты, мастер-классы)</t>
+        </is>
+      </c>
+      <c r="F5" s="18" t="inlineStr">
+        <is>
+          <t>2
+(Рекомендован)</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>• Профильное историческое образование (ВШЭ)
+• Высокая личная осознанная мотивация
+• Свободный график (32 ч/мес при норме 16 ч)
+• Готовность к сменам в выходные</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="inlineStr">
+        <is>
+          <t>• Сессионные пики 1 курса (декабрь–январь, июнь): риск временного снижения активности во время экзаменов.</t>
+        </is>
+      </c>
+      <c r="I5" s="6" t="inlineStr">
+        <is>
+          <t>1. «Как у вас устроена зимняя сессия в Вышке и сможете ли вы дежурить на новогодних музейных программах в начале января?»
+2. «Какой исторический период вам ближе для разработки интерактивов — Смутное время или более поздние эпохи?»</t>
+        </is>
+      </c>
+      <c r="J5" s="6" t="inlineStr">
+        <is>
+          <t>Снятие слепого штрафа за 1 курс: часы подтверждены (32 ч/мес) -&gt; давать балл 2, а не снижать оценку.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="290" customHeight="1">
+      <c r="A6" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>Работающий специалист
+(Образцовый кандидат под выходные)</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>Константин Мельников, 29 лет
+Работаю (IT-инженер)
+МАИ (специалитет, окончен)</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>1. Согласие на ОПД: Да, даю согласие
+2. ФИО: Мельников Константин Андреевич
+3. Электронная почта: melnikov.k.it@yandex.ru
+4. Ссылка на страницу ВК: https://vk.com/kostya_melnikov_tech
+5. Дата рождения: 12.04.1997 (29 лет)
+6. Ваш нынешний статус: Работаю
+7. ВУЗ: Другое
+8. ВУЗ (Другое): Московский авиационный институт (МАИ)
+9. Факультет: Институт информационных систем и технологий
+10. Курс: Окончил специалитет (2020 г.)
+11. Сфера научных интересов: Военная история России XVIII–XX веков, фортификация, история артиллерии
+12. Опыт работы, стажировки, проекты: Ведущий IT-инженер с гибким графиком. Опыт тимлида волонтёров на Московском марафоне и фестивале «Круг света» (навигация потоков до 10 000 чел, решение конфликтных ситуаций, инструктаж волонтёров).
+13. Иностранные языки (B1 и выше): Английский язык (B2)
+14. Почему Вы выбрали волонтёрскую программу Исторического музея?: Всю рабочую неделю сижу за компьютером, в выходные хочу живого общения с людьми и культурой. Обожаю военную историю России и хочу быть надёжной опорой для музейных событий.
+15. Чего Вы ожидаете от волонтёрства в Историческом музее?: Координация навигации на масштабных фестивалях («Ночь музеев», исторические праздники), управление потоками гостей, помощь старшим кураторам.
+16. Сколько времени Вы готовы уделять добровольческой деятельности в месяц?: 28 часов в месяц (каждые суббота и воскресенье полностью свободны, готов к длинным сменам по 7-8 часов).
+17. Ваши хобби: Стендовый моделизм военной техники, бег на длинные дистанции, посещение исторических выставок
+18. В работу какого направления Вы бы хотели включиться?: Организационное направление (помощь в организации культурно-массовых мероприятий)
+19. Откуда Вы узнали о Волонтерской программе?: Социальные сети</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>Организационное направление
+(навигация, координация)</t>
+        </is>
+      </c>
+      <c r="F6" s="19" t="inlineStr">
+        <is>
+          <t>3
+(Хорошая анкета)</t>
+        </is>
+      </c>
+      <c r="G6" s="9" t="inlineStr">
+        <is>
+          <t>• Оконченное образование, бытовая стабильность
+• Подтверждённый опыт координации людей в толпе (тимлид)
+• Идеальное совпадение свободного времени (выходные) с пиковыми событиями музея (28 ч/мес)
+• Отсутствие сессий</t>
+        </is>
+      </c>
+      <c r="H6" s="9" t="inlineStr">
+        <is>
+          <t>• Будни с 9 до 18 заблокированы работой (не подходит для будничных фондов, но идеален для фестивалей в выходные).</t>
+        </is>
+      </c>
+      <c r="I6" s="9" t="inlineStr">
+        <is>
+          <t>1. «Большинство масштабных событий проходит по субботам и вечерам пятниц. Готовы ли вы координировать команду навигаторов в дни выставочных пиков?»
+2. «Был ли у вас опыт разрешения сложных конфликтных ситуаций с гостями на прошлых мероприятиях?»</t>
+        </is>
+      </c>
+      <c r="J6" s="9" t="inlineStr">
+        <is>
+          <t>Эталонный балл 3: зрелый кандидат, опыт тимлида, высокая стабильность и готовность к сменам выходного дня.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="290" customHeight="1">
+      <c r="A7" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Неопределившийся кандидат
+(Маршрутизация смешанного трека)</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>Анна Григорьева, 20 лет
+Студентка (очно), 2 курс
+РГГУ (Культурология)</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>1. Согласие на ОПД: Да, даю согласие
+2. ФИО: Григорьева Анна Сергеевна
+3. Электронная почта: anya.grigorieva2006@mail.ru
+4. Ссылка на страницу ВК: https://vk.com/anya_grig_art
+5. Дата рождения: 28.05.2006 (20 лет)
+6. Ваш нынешний статус: Студент
+7. ВУЗ: Российский государственный гуманитарный университет (РГГУ)
+8. ВУЗ (Другое): —
+9. Факультет: Факультет культурологии
+10. Курс: 2 курс бакалавриата
+11. Сфера научных интересов: История повседневности Москвы конца XIX века, история моды и костюма
+12. Опыт работы, стажировки, проекты: Помощь на студенческой межвузовской конференции (встреча и регистрация участников, фотосъёмка для паблика факультета). В музеях ранее не волонтёрила.
+13. Иностранные языки (B1 и выше): Английский язык (B1)
+14. Почему Вы выбрали волонтёрскую программу Исторического музея?: Очень люблю экспозицию Исторического музея на Красной площади, часто посещаю временные выставки. Хочу заглянуть во внутреннюю жизнь музея и стать полезной.
+15. Чего Вы ожидаете от волонтёрства в Историческом музее?: Хочу попробовать разные задачи — и в залах с посетителями, и в создании контента/фото для соцсетей, чтобы понять, какое направление мне ближе всего.
+16. Сколько времени Вы готовы уделять добровольческой деятельности в месяц?: 16–20 часов в месяц (свободна во второй половине пятницы и в субботу).
+17. Ваши хобби: Фотография архитектуры и выставок, ведение культурного телеграм-канала, рисование скетчей
+18. В работу какого направления Вы бы хотели включиться?: Пока не определился
+19. Откуда Вы узнали о Волонтерской программе?: Рекомендации друзей</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>Медиа / Организационное
+(рекомендован смешанный трек)</t>
+        </is>
+      </c>
+      <c r="F7" s="18" t="inlineStr">
+        <is>
+          <t>ТРЕБУЕТ ПРОВЕРКИ
+(между 1 и 2)</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>• Профильный культурологический кругозор
+• Искренний интерес к ГИМ
+• Базовые навыки фотосъёмки и коммуникации
+• Достаточный запас времени (16–20 ч/мес)</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>• Размытые ожидания («хочу всего понемногу»).
+• Риск быстрой потери интереса при встрече с рутиной без чёткой цели.</t>
+        </is>
+      </c>
+      <c r="I7" s="6" t="inlineStr">
+        <is>
+          <t>1. «Что вам ближе для первого шага: подготовить фоторепортаж/пост для соцсетей или встречать гостей в залах в выходной?»
+2. «Готовы ли вы включиться в одну разовую акцию в выходной день, чтобы познакомиться с кураторами и определиться с постоянным треком?»</t>
+        </is>
+      </c>
+      <c r="J7" s="6" t="inlineStr">
+        <is>
+          <t>Маршрутизация 'Пока не определился': система не ставит случайный балл, а выставляет статус 'требует проверки' и предлагает смешанный трек.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="290" customHeight="1">
+      <c r="A8" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>Опытный перегруженный волонтёр
+(Критический дефицит часов)</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>Виктория Белова, 21 год
+Студентка (очно), 3 курс
+МГУ им. Ломоносова (Истфак)</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>1. Согласие на ОПД: Да, даю согласие
+2. ФИО: Белова Виктория Павловна
+3. Электронная почта: vika.belova.history@gmail.com
+4. Ссылка на страницу ВК: https://vk.com/vika_culture_pro
+5. Дата рождения: 03.11.2004 (21 год)
+6. Ваш нынешний статус: Студент
+7. ВУЗ: МГУ имени М.В. Ломоносова
+8. ВУЗ (Другое): —
+9. Факультет: Исторический факультет
+10. Курс: 3 курс бакалавриата
+11. Сфера научных интересов: Музеология, дворянская усадебная культура, атрибуция предметов быта
+12. Опыт работы, стажировки, проекты: Волонтёр Государственной Третьяковской галереи (дежурства каждую субботу в Лаврушинском), волонтёр Музея Москвы, руководитель пресс-службы Студсовета истфака МГУ.
+13. Иностранные языки (B1 и выше): Английский язык (C1), Французский язык (B1)
+14. Почему Вы выбрали волонтёрскую программу Исторического музея?: ГИМ — центральный исторический музей России. Хочу войти в волонтёрский актив и применить свой обширный практический опыт организации мероприятий и квестов.
+15. Чего Вы ожидаете от волонтёрства в Историческом музее?: Работы исключительно в фондах музея с подлинными коллекциями.
+16. Сколько времени Вы готовы уделять добровольческой деятельности в месяц?: 4 часа в месяц (все субботы и воскресенья заняты сменами в Третьяковке, четверги — собрания студсовета, будни — очные пары до 17:00. Смогу выделить максимум 1 вечер в месяц).
+17. Ваши хобби: Посещение вернисажей, академический вокал, написание статей об искусстве
+18. В работу какого направления Вы бы хотели включиться?: Фондовое направление
+19. Откуда Вы узнали о Волонтерской программе?: Социальные сети</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>Не рекомендован
+(Отказ на скрининге)</t>
+        </is>
+      </c>
+      <c r="F8" s="20" t="inlineStr">
+        <is>
+          <t>0
+(Не позвали на очное)</t>
+        </is>
+      </c>
+      <c r="G8" s="9" t="inlineStr">
+        <is>
+          <t>• Профессиональный опыт в ведущих музеях Москвы
+• Развитые лидерские и организаторские навыки
+• Знание музейного этикета</t>
+        </is>
+      </c>
+      <c r="H8" s="9" t="inlineStr">
+        <is>
+          <t>• КРИТИЧЕСКИЙ ДЕФИЦИТ ЧАСОВ: доступно всего 4 ч/мес (норматив ГИМ от 16 ч/мес)!
+• Мультиволонтёрство: субботы и воскресенья заняты Третьяковкой.
+• Конфликт графика: выбраны фонды (будни 10-18), но в будни очные пары до вечера.</t>
+        </is>
+      </c>
+      <c r="I8" s="9" t="inlineStr">
+        <is>
+          <t>Очное интервью не назначается. В случае обращения куратор может уточнить:
+«Готовы ли вы освободить субботы в Третьяковке и гарантировать минимум 16 часов в месяц для ГИМ?»</t>
+        </is>
+      </c>
+      <c r="J8" s="9" t="inlineStr">
+        <is>
+          <t>Отказ на скрининге (Балл 0): несмотря на богатое резюме, невыполнение норматива часов (4 ч &lt; 16 ч) и конфликт расписания делают участие невозможным.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1020,7 +1475,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1244,13 +1699,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1598,12 +2053,54 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" s="14" t="inlineStr">
+        <is>
+          <t>ЧТО СЧИТАЕТСЯ ПОЛЕЗНОЙ РЕКОМЕНДАЦИЕЙ ДЛЯ КУРАТОРА ГИМ (требования заказчика):</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="15" t="inlineStr">
+        <is>
+          <t>1. Объяснимый кураторский балл (0–3) либо пометка «требует проверки» при пограничных данных (не подбирать произвольно).</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="15" t="inlineStr">
+        <is>
+          <t>2. Точное рекомендуемое направление с учётом совместимости графика кандидата (например, очников не отправлять в будничные фонды).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="15" t="inlineStr">
+        <is>
+          <t>3. Блок «Возможные проблемы» (Риски): ранняя детекция скрытых конфликтов (накладка сессий, очные пары, мультиволонтёрство, скрытый поиск работы).</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="15" t="inlineStr">
+        <is>
+          <t>4. 1–2 целевых вопроса для очного интервью, бьющих точно в выявленные риски или неопределённости кандидата (экономит 20–30 мин на встрече).</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="15" t="inlineStr">
+        <is>
+          <t>5. Тестовые сценарии для калибровки оценщика: см. лист «4 Контрастных сценария» в этом файле (4 полярных кейса с полными 19 ответами).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
docs: add GIM contrast scenarios and synthetic candidates spreadsheets
</commit_message>
<xml_diff>
--- a/docs/Критерии_отбора_ГИМ.xlsx
+++ b/docs/Критерии_отбора_ГИМ.xlsx
@@ -8,11 +8,10 @@
   </bookViews>
   <sheets>
     <sheet name="5 Критериев отбора" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="4 Контрастных сценария" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Шкала оценок кураторов 0-3" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Направления ГИМ" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Формат выгрузки для куратора" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Объективные фильтры" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Шкала оценок кураторов 0-3" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Направления ГИМ" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Формат выгрузки для куратора" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Объективные фильтры" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="12">
+  <fonts count="19">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -94,8 +93,50 @@
       <color rgb="00C00000"/>
       <sz val="12"/>
     </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="008B181B"/>
+      <sz val="15"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <i val="1"/>
+      <color rgb="00555555"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00004085"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <color rgb="00000000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="000056B3"/>
+      <sz val="10"/>
+      <u val="single"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -132,8 +173,35 @@
         <bgColor rgb="00C00000"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00CCE5FF"/>
+        <bgColor rgb="00CCE5FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="008B181B"/>
+        <bgColor rgb="008B181B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D4EDDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF3CD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8D7DA"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -155,11 +223,26 @@
         <color rgb="00D9D9D9"/>
       </bottom>
     </border>
+    <border/>
+    <border>
+      <left style="thin">
+        <color rgb="00CCCCCC"/>
+      </left>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -211,6 +294,42 @@
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="9" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="10" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="11" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -600,7 +719,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Сверено с ТЗ и ответами ГИМ (21.10.2026). 4 эталонных тестовых сценария: см. лист «4 Контрастных сценария»</t>
+          <t>Сверено с ТЗ и ответами ГИМ (21.10.2026). Тестовые полигоны: docs/Контрастные_сценарии_ГИМ.xlsx (4 ключевых кейса) и docs/Синтетические_кандидаты_ГИМ.xlsx (12 персон)</t>
         </is>
       </c>
     </row>
@@ -889,408 +1008,6 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:J8"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="52" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="28" customWidth="1" min="7" max="7"/>
-    <col width="30" customWidth="1" min="8" max="8"/>
-    <col width="36" customWidth="1" min="9" max="9"/>
-    <col width="30" customWidth="1" min="10" max="10"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Государственный исторический музей (ГИМ) · 4 Контрастных сценария: распределение оценок [0, 2, 3, ТРЕБУЕТ ПРОВЕРКИ]</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Полные ответы на ВСЕ 19 вопросов анкеты ГИМ. Чёткое распределение: один с 0, один с 2, один с 3 и один со статусом ТРЕБУЕТ ПРОВЕРКИ. 21.10.2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="28" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>№</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Тип сценария</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>Кандидат и статус</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>ПОЛНЫЕ ВХОДНЫЕ ОТВЕТЫ НА ВСЕ 19 ВОПРОСОВ АНКЕТЫ ГИМ</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>Ожидаемое направление</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>Кураторский балл</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>Сильные стороны</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>Возможные проблемы (Риски)</t>
-        </is>
-      </c>
-      <c r="I4" s="3" t="inlineStr">
-        <is>
-          <t>Ожидаемые вопросы для интервью</t>
-        </is>
-      </c>
-      <c r="J4" s="3" t="inlineStr">
-        <is>
-          <t>Что проверяет кейс</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="290" customHeight="1">
-      <c r="A5" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>Мотивированный первокурсник
-(Исключение по нагрузке)</t>
-        </is>
-      </c>
-      <c r="C5" s="6" t="inlineStr">
-        <is>
-          <t>Алексей Смирнов, 18 лет
-Студент (очно), 1 курс
-НИУ ВШЭ (История)</t>
-        </is>
-      </c>
-      <c r="D5" s="6" t="inlineStr">
-        <is>
-          <t>1. Согласие на ОПД: Да, даю согласие
-2. ФИО: Смирнов Алексей Дмитриевич
-3. Электронная почта: smirnov.alex.hse@gmail.com
-4. Ссылка на страницу ВК: https://vk.com/smirnov_alex_hse
-5. Дата рождения: 15.09.2008 (18 лет)
-6. Ваш нынешний статус: Студент
-7. ВУЗ: Национальный исследовательский университет «Высшая школа экономики» (НИУ ВШЭ)
-8. ВУЗ (Другое): —
-9. Факультет: Факультет гуманитарных наук, ОП «История»
-10. Курс: 1 курс бакалавриата
-11. Сфера научных интересов: История России XVII века, Смутное время, формирование сословий
-12. Опыт работы, стажировки, проекты: Волонтёр школьных исторических чтений, проведение Дня открытых дверей в лицее ВШЭ (навигация гостей, регистрация участников)
-13. Иностранные языки (B1 и выше): Английский язык (B2)
-14. Почему Вы выбрали волонтёрскую программу Исторического музея?: С детства посещаю ГИМ. Для меня ГИМ — это главный музей страны по профилю моего исторического образования. Хочу быть полезным музею и развиваться в музейной среде.
-15. Чего Вы ожидаете от волонтёрства в Историческом музее?: Применить академические знания на практике, научиться работать с аудиторией, участвовать в проведении квестов и интерактивов для подростков.
-16. Сколько времени Вы готовы уделять добровольческой деятельности в месяц?: 32 часа в месяц (обучаюсь по индивидуальному плану: вторник и четверг без пар, все выходные свободны. Других проектов нет).
-17. Ваши хобби: Настольные исторические стратегии, чтение архивных мемуаров, походы в музеи
-18. В работу какого направления Вы бы хотели включиться?: Проектное направление (разработка квестов/мастер-классов для культурно-массовых мероприятий)
-19. Откуда Вы узнали о Волонтерской программе?: Сайт Исторического музея</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>Проектное направление
-(квесты, мастер-классы)</t>
-        </is>
-      </c>
-      <c r="F5" s="18" t="inlineStr">
-        <is>
-          <t>2
-(Рекомендован)</t>
-        </is>
-      </c>
-      <c r="G5" s="6" t="inlineStr">
-        <is>
-          <t>• Профильное историческое образование (ВШЭ)
-• Высокая личная осознанная мотивация
-• Свободный график (32 ч/мес при норме 16 ч)
-• Готовность к сменам в выходные</t>
-        </is>
-      </c>
-      <c r="H5" s="6" t="inlineStr">
-        <is>
-          <t>• Сессионные пики 1 курса (декабрь–январь, июнь): риск временного снижения активности во время экзаменов.</t>
-        </is>
-      </c>
-      <c r="I5" s="6" t="inlineStr">
-        <is>
-          <t>1. «Как у вас устроена зимняя сессия в Вышке и сможете ли вы дежурить на новогодних музейных программах в начале января?»
-2. «Какой исторический период вам ближе для разработки интерактивов — Смутное время или более поздние эпохи?»</t>
-        </is>
-      </c>
-      <c r="J5" s="6" t="inlineStr">
-        <is>
-          <t>Снятие слепого штрафа за 1 курс: часы подтверждены (32 ч/мес) -&gt; давать балл 2, а не снижать оценку.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="290" customHeight="1">
-      <c r="A6" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="B6" s="8" t="inlineStr">
-        <is>
-          <t>Работающий специалист
-(Образцовый кандидат под выходные)</t>
-        </is>
-      </c>
-      <c r="C6" s="9" t="inlineStr">
-        <is>
-          <t>Константин Мельников, 29 лет
-Работаю (IT-инженер)
-МАИ (специалитет, окончен)</t>
-        </is>
-      </c>
-      <c r="D6" s="9" t="inlineStr">
-        <is>
-          <t>1. Согласие на ОПД: Да, даю согласие
-2. ФИО: Мельников Константин Андреевич
-3. Электронная почта: melnikov.k.it@yandex.ru
-4. Ссылка на страницу ВК: https://vk.com/kostya_melnikov_tech
-5. Дата рождения: 12.04.1997 (29 лет)
-6. Ваш нынешний статус: Работаю
-7. ВУЗ: Другое
-8. ВУЗ (Другое): Московский авиационный институт (МАИ)
-9. Факультет: Институт информационных систем и технологий
-10. Курс: Окончил специалитет (2020 г.)
-11. Сфера научных интересов: Военная история России XVIII–XX веков, фортификация, история артиллерии
-12. Опыт работы, стажировки, проекты: Ведущий IT-инженер с гибким графиком. Опыт тимлида волонтёров на Московском марафоне и фестивале «Круг света» (навигация потоков до 10 000 чел, решение конфликтных ситуаций, инструктаж волонтёров).
-13. Иностранные языки (B1 и выше): Английский язык (B2)
-14. Почему Вы выбрали волонтёрскую программу Исторического музея?: Всю рабочую неделю сижу за компьютером, в выходные хочу живого общения с людьми и культурой. Обожаю военную историю России и хочу быть надёжной опорой для музейных событий.
-15. Чего Вы ожидаете от волонтёрства в Историческом музее?: Координация навигации на масштабных фестивалях («Ночь музеев», исторические праздники), управление потоками гостей, помощь старшим кураторам.
-16. Сколько времени Вы готовы уделять добровольческой деятельности в месяц?: 28 часов в месяц (каждые суббота и воскресенье полностью свободны, готов к длинным сменам по 7-8 часов).
-17. Ваши хобби: Стендовый моделизм военной техники, бег на длинные дистанции, посещение исторических выставок
-18. В работу какого направления Вы бы хотели включиться?: Организационное направление (помощь в организации культурно-массовых мероприятий)
-19. Откуда Вы узнали о Волонтерской программе?: Социальные сети</t>
-        </is>
-      </c>
-      <c r="E6" s="8" t="inlineStr">
-        <is>
-          <t>Организационное направление
-(навигация, координация)</t>
-        </is>
-      </c>
-      <c r="F6" s="19" t="inlineStr">
-        <is>
-          <t>3
-(Хорошая анкета)</t>
-        </is>
-      </c>
-      <c r="G6" s="9" t="inlineStr">
-        <is>
-          <t>• Оконченное образование, бытовая стабильность
-• Подтверждённый опыт координации людей в толпе (тимлид)
-• Идеальное совпадение свободного времени (выходные) с пиковыми событиями музея (28 ч/мес)
-• Отсутствие сессий</t>
-        </is>
-      </c>
-      <c r="H6" s="9" t="inlineStr">
-        <is>
-          <t>• Будни с 9 до 18 заблокированы работой (не подходит для будничных фондов, но идеален для фестивалей в выходные).</t>
-        </is>
-      </c>
-      <c r="I6" s="9" t="inlineStr">
-        <is>
-          <t>1. «Большинство масштабных событий проходит по субботам и вечерам пятниц. Готовы ли вы координировать команду навигаторов в дни выставочных пиков?»
-2. «Был ли у вас опыт разрешения сложных конфликтных ситуаций с гостями на прошлых мероприятиях?»</t>
-        </is>
-      </c>
-      <c r="J6" s="9" t="inlineStr">
-        <is>
-          <t>Эталонный балл 3: зрелый кандидат, опыт тимлида, высокая стабильность и готовность к сменам выходного дня.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="290" customHeight="1">
-      <c r="A7" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>Неопределившийся кандидат
-(Маршрутизация смешанного трека)</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>Анна Григорьева, 20 лет
-Студентка (очно), 2 курс
-РГГУ (Культурология)</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>1. Согласие на ОПД: Да, даю согласие
-2. ФИО: Григорьева Анна Сергеевна
-3. Электронная почта: anya.grigorieva2006@mail.ru
-4. Ссылка на страницу ВК: https://vk.com/anya_grig_art
-5. Дата рождения: 28.05.2006 (20 лет)
-6. Ваш нынешний статус: Студент
-7. ВУЗ: Российский государственный гуманитарный университет (РГГУ)
-8. ВУЗ (Другое): —
-9. Факультет: Факультет культурологии
-10. Курс: 2 курс бакалавриата
-11. Сфера научных интересов: История повседневности Москвы конца XIX века, история моды и костюма
-12. Опыт работы, стажировки, проекты: Помощь на студенческой межвузовской конференции (встреча и регистрация участников, фотосъёмка для паблика факультета). В музеях ранее не волонтёрила.
-13. Иностранные языки (B1 и выше): Английский язык (B1)
-14. Почему Вы выбрали волонтёрскую программу Исторического музея?: Очень люблю экспозицию Исторического музея на Красной площади, часто посещаю временные выставки. Хочу заглянуть во внутреннюю жизнь музея и стать полезной.
-15. Чего Вы ожидаете от волонтёрства в Историческом музее?: Хочу попробовать разные задачи — и в залах с посетителями, и в создании контента/фото для соцсетей, чтобы понять, какое направление мне ближе всего.
-16. Сколько времени Вы готовы уделять добровольческой деятельности в месяц?: 16–20 часов в месяц (свободна во второй половине пятницы и в субботу).
-17. Ваши хобби: Фотография архитектуры и выставок, ведение культурного телеграм-канала, рисование скетчей
-18. В работу какого направления Вы бы хотели включиться?: Пока не определился
-19. Откуда Вы узнали о Волонтерской программе?: Рекомендации друзей</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>Медиа / Организационное
-(рекомендован смешанный трек)</t>
-        </is>
-      </c>
-      <c r="F7" s="18" t="inlineStr">
-        <is>
-          <t>ТРЕБУЕТ ПРОВЕРКИ
-(между 1 и 2)</t>
-        </is>
-      </c>
-      <c r="G7" s="6" t="inlineStr">
-        <is>
-          <t>• Профильный культурологический кругозор
-• Искренний интерес к ГИМ
-• Базовые навыки фотосъёмки и коммуникации
-• Достаточный запас времени (16–20 ч/мес)</t>
-        </is>
-      </c>
-      <c r="H7" s="6" t="inlineStr">
-        <is>
-          <t>• Размытые ожидания («хочу всего понемногу»).
-• Риск быстрой потери интереса при встрече с рутиной без чёткой цели.</t>
-        </is>
-      </c>
-      <c r="I7" s="6" t="inlineStr">
-        <is>
-          <t>1. «Что вам ближе для первого шага: подготовить фоторепортаж/пост для соцсетей или встречать гостей в залах в выходной?»
-2. «Готовы ли вы включиться в одну разовую акцию в выходной день, чтобы познакомиться с кураторами и определиться с постоянным треком?»</t>
-        </is>
-      </c>
-      <c r="J7" s="6" t="inlineStr">
-        <is>
-          <t>Маршрутизация 'Пока не определился': система не ставит случайный балл, а выставляет статус 'требует проверки' и предлагает смешанный трек.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="290" customHeight="1">
-      <c r="A8" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="B8" s="8" t="inlineStr">
-        <is>
-          <t>Опытный перегруженный волонтёр
-(Критический дефицит часов)</t>
-        </is>
-      </c>
-      <c r="C8" s="9" t="inlineStr">
-        <is>
-          <t>Виктория Белова, 21 год
-Студентка (очно), 3 курс
-МГУ им. Ломоносова (Истфак)</t>
-        </is>
-      </c>
-      <c r="D8" s="9" t="inlineStr">
-        <is>
-          <t>1. Согласие на ОПД: Да, даю согласие
-2. ФИО: Белова Виктория Павловна
-3. Электронная почта: vika.belova.history@gmail.com
-4. Ссылка на страницу ВК: https://vk.com/vika_culture_pro
-5. Дата рождения: 03.11.2004 (21 год)
-6. Ваш нынешний статус: Студент
-7. ВУЗ: МГУ имени М.В. Ломоносова
-8. ВУЗ (Другое): —
-9. Факультет: Исторический факультет
-10. Курс: 3 курс бакалавриата
-11. Сфера научных интересов: Музеология, дворянская усадебная культура, атрибуция предметов быта
-12. Опыт работы, стажировки, проекты: Волонтёр Государственной Третьяковской галереи (дежурства каждую субботу в Лаврушинском), волонтёр Музея Москвы, руководитель пресс-службы Студсовета истфака МГУ.
-13. Иностранные языки (B1 и выше): Английский язык (C1), Французский язык (B1)
-14. Почему Вы выбрали волонтёрскую программу Исторического музея?: ГИМ — центральный исторический музей России. Хочу войти в волонтёрский актив и применить свой обширный практический опыт организации мероприятий и квестов.
-15. Чего Вы ожидаете от волонтёрства в Историческом музее?: Работы исключительно в фондах музея с подлинными коллекциями.
-16. Сколько времени Вы готовы уделять добровольческой деятельности в месяц?: 4 часа в месяц (все субботы и воскресенья заняты сменами в Третьяковке, четверги — собрания студсовета, будни — очные пары до 17:00. Смогу выделить максимум 1 вечер в месяц).
-17. Ваши хобби: Посещение вернисажей, академический вокал, написание статей об искусстве
-18. В работу какого направления Вы бы хотели включиться?: Фондовое направление
-19. Откуда Вы узнали о Волонтерской программе?: Социальные сети</t>
-        </is>
-      </c>
-      <c r="E8" s="8" t="inlineStr">
-        <is>
-          <t>Не рекомендован
-(Отказ на скрининге)</t>
-        </is>
-      </c>
-      <c r="F8" s="20" t="inlineStr">
-        <is>
-          <t>0
-(Не позвали на очное)</t>
-        </is>
-      </c>
-      <c r="G8" s="9" t="inlineStr">
-        <is>
-          <t>• Профессиональный опыт в ведущих музеях Москвы
-• Развитые лидерские и организаторские навыки
-• Знание музейного этикета</t>
-        </is>
-      </c>
-      <c r="H8" s="9" t="inlineStr">
-        <is>
-          <t>• КРИТИЧЕСКИЙ ДЕФИЦИТ ЧАСОВ: доступно всего 4 ч/мес (норматив ГИМ от 16 ч/мес)!
-• Мультиволонтёрство: субботы и воскресенья заняты Третьяковкой.
-• Конфликт графика: выбраны фонды (будни 10-18), но в будни очные пары до вечера.</t>
-        </is>
-      </c>
-      <c r="I8" s="9" t="inlineStr">
-        <is>
-          <t>Очное интервью не назначается. В случае обращения куратор может уточнить:
-«Готовы ли вы освободить субботы в Третьяковке и гарантировать минимум 16 часов в месяц для ГИМ?»</t>
-        </is>
-      </c>
-      <c r="J8" s="9" t="inlineStr">
-        <is>
-          <t>Отказ на скрининге (Балл 0): несмотря на богатое резюме, невыполнение норматива часов (4 ч &lt; 16 ч) и конфликт расписания делают участие невозможным.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1475,7 +1192,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1699,7 +1416,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2091,7 +1808,7 @@
     <row r="22">
       <c r="A22" s="15" t="inlineStr">
         <is>
-          <t>5. Тестовые сценарии для калибровки оценщика: см. лист «4 Контрастных сценария» в этом файле (4 полярных кейса с полными 19 ответами).</t>
+          <t>5. Тестовые полигоны для калибровки: docs/Контрастные_сценарии_ГИМ.xlsx (4 контрастных случая) и docs/Синтетические_кандидаты_ГИМ.xlsx (12 кандидатов со всеми 19 ответами).</t>
         </is>
       </c>
     </row>
@@ -2100,7 +1817,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
docs: update GIM selection criteria and Eva expert expectations spreadsheets
</commit_message>
<xml_diff>
--- a/docs/Критерии_отбора_ГИМ.xlsx
+++ b/docs/Критерии_отбора_ГИМ.xlsx
@@ -787,10 +787,10 @@
         <is>
           <t>• Шаблонные отписки, общие фразы или отсутствие ответов
 • Не объясняет выбор именно ГИМ
-• Жёсткая фиксация ТОЛЬКО на фондах: в фонд мало мест, риск «мёртвой души» при отказе
+• Выбор исключительно фондового направления при отсутствии опыта (в фондах мало мест, риск невостребованности при отказе)
 • Скрытый поиск работы («с перспективой трудоустройства»)
 • Административное принуждение («сказали в вузе ради практики»)
-• Несовпадение сферы интересов с музеем</t>
+• Несовпадение сферы интересов с музейной тематикой</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
@@ -875,41 +875,36 @@
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>• Оконченное образование (бакалавриат завершён, человек не учится, стабильный график)
-• Старшие курсы (от 2 курса бакалавриата, магистратура) — выше осознанность и научные интересы
-• Наличие свободного времени (от 16 часов в месяц)
-• Готовность к сменам в выходные дни и вечерами</t>
+          <t>• Достаточное количество времени: готовность уделять от 16 часов в месяц (положительный ориентир регулярности)
+• Стабильный график участия
+• Совпадение графика с мероприятиями музея: готовность к вечерним сменам или выходным дням</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>• ⚠️ Высокая загруженность: совмещение учёбы на очном отделении с работой на полную ставку
-• ⚠️ 1-й курс бакалавриата: риск нехватки опыта и выгорания в первую сессию
-• ⚠️ Блокировка будней: очное обучение не позволяет работать в фондах (будни 10:00–18:00)
-• ⚠️ Множественное волонтёрство прямо сейчас (участие в 2+ других музеях/программах)</t>
+          <t>• Заявлено мало часов в месяц (гипотеза о риске недостаточной регулярности, требует проверки задач направления)
+• Несовпадение очного обучения с дневным графиком фондов (при отсутствии подтверждённых свободных дней)
+• Полная занятость (работа 5/2) без подтверждённой готовности участвовать в событиях выходного дня
+• Риск экзаменационных сессий: не подтверждена регулярность смен в период зачётов</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>• ТРЕБОВАНИЕ ЗАКАЗЧИКА (21.10.2026): предпочтительны свободные кандидаты, НО ВОЗМОЖНЫ ИСКЛЮЧЕНИЯ!
-• ❌ ЗАПРЕЩЕНО автоматически отсеивать очников, первокурсников или работающих!
-• ПРАВИЛО ИСКЛЮЧЕНИЯ: проверять реальный график. Если очник/работающий готов выходить в выходные на проекты/орг — давать зелёный свет</t>
+          <t>• Приоритет реальной подтверждённой доступности, а не формального статуса
+• Работа 5/2 НЕ означает отказ, если кандидат свободен в сб/вс для проведения мероприятий
+• Правило: возможность участия очников в дневных сменах фондов требует обязательного уточнения расписания пар</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>Саммари: «Доступность: высокая / средняя / ограниченная».
-Возможные проблемы:
-«Конфликт расписания (очник претендует на фонды)»
-«Риск дефицита часов в сессию (1 курс)»
-«Параллельные проекты».</t>
+          <t>Саммари: «Доступность: подтверждена / требует согласования».
+Возможная проблема: «Очное обучение: требует согласования с графиком фондовых отделов» или «Работа 5/2: ориентир на сб/вс».</t>
         </is>
       </c>
       <c r="G7" s="6" t="inlineStr">
         <is>
-          <t>• Занятость: «Сколько времени вы готовы уделять: от 16 ч/мес? Предпочитаете регулярный график или гибкий?»
-• Конфликт фондов: «Фонды открыты только по будням 10–18. Сможете присутствовать в эти часы или выберем трек с дежурствами в выходные?»
-• «Состоите ли вы в других волонтёрских организациях?»</t>
+          <t>• «В какие дни недели и часы вам удобнее участвовать в волонтёрских сменах?»
+• «Готовы ли вы помогать в выходные дни на выставочных проектах и фестивалях?»</t>
         </is>
       </c>
     </row>
@@ -932,10 +927,9 @@
       </c>
       <c r="D8" s="9" t="inlineStr">
         <is>
-          <t>• Полупустая или пустая анкета («телеграфный стиль», отписки по 1 слову)
-• Некорректная ссылка на страницу ВК или указан только телефон
-• Закрытый профиль ВК (сложно оперативно связаться кураторам)
-• Пустая страница ВК без признаков активности</t>
+          <t>• Первый курс бакалавриата (период адаптации к вузу, риск нестабильного графика в первую сессию)
+• Студенты выпускных курсов (4 курс бакалавриата) в период подготовки диплома (май-июнь)
+• Некорректная ссылка на контакт либо невозможность оперативной связи с кандидатом</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -947,14 +941,14 @@
       </c>
       <c r="F8" s="9" t="inlineStr">
         <is>
-          <t>Саммари: «Качество заполнения анкеты: высокое / среднее / низкое».
-Возможная проблема: «Закрытый профиль VK — требуется подтвердить альтернативный контакт».</t>
+          <t>Саммари: «Статус: студент (курс) / работающий / выпускник».
+Возможная проблема: «1 курс бакалавриата: риск адаптации» или «Выпускной курс: дипломная нагрузка».</t>
         </is>
       </c>
       <c r="G8" s="9" t="inlineStr">
         <is>
-          <t>• Канал связи: «Взаимодействие с волонтёрами ГИМ ведётся на базе ВКонтакте. Будет ли у вас возможность оперативно быть на связи в беседах VK?»
-• «Готовы ли вы открыть ЛС для куратора программы?»</t>
+          <t>• Для 1 курса бакалавриата: «Как вы планируете распределять нагрузку между учёбой и волонтёрством?»
+• Для выпускников: «Потребуется ли вам перерыв на подготовку диплома?»</t>
         </is>
       </c>
     </row>
@@ -1033,7 +1027,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Утверждено заказчиком 21.10.2026: приоритеты выводятся из практики кураторов, а не назначаются произвольно</t>
+          <t>Экспертная модель команды на основе исторической практики кураторов ГИМ (2024–2025). Ориентир для содержательного анализа, не является утверждённым музеем автоматическим регламентом.</t>
         </is>
       </c>
     </row>
@@ -1086,12 +1080,12 @@
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>Отказ на этапе скрининга (Не рекомендован)</t>
+          <t>Исторический статус: не приглашён на очное собеседование (в системе: сигнал куратору о факторах риска)</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>Анкета отправляется в архив с указанием причины отказа (объективное несоответствие требованиям программы).</t>
+          <t>Куратор проверяет объективные барьеры (возраст до 18 лет, отсутствие согласия ОПД, невозможность связи) либо передаёт карточку на ручное рассмотрение.</t>
         </is>
       </c>
     </row>
@@ -1109,8 +1103,8 @@
       <c r="C6" s="9" t="inlineStr">
         <is>
           <t>• Лаконичные ответы (1–2 слова), шаблонные фразы («опыт», «интересно»)
-• Не указан опыт и нет конкретики, чем кандидат может помочь музею
-• Закрытый профиль ВК, пустая страница
+• В анкете не описан опыт и нет конкретики, чем кандидат может помочь музею
+• Не указан канал оперативной связи или контакт недоступен
 • Высокий риск перегрузки (1 курс + работа + другие проекты) без подтверждения доступности часов</t>
         </is>
       </c>
@@ -1169,11 +1163,11 @@
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>• Развёрнутые, глубокие ответы, искренний интерес к ГИМ и истории
+          <t>• Развёрнутые, осознанные ответы, устойчивый интерес к ГИМ и истории
 • Профильный опыт (архивы, фонды, инклюзия, координация мероприятий, медиа/дизайн) либо дефицитная специальность (дефектология, сурдокоммуникация)
-• Прозрачный цифровой след, открытый ВК
+• Подтверждённый контакт для связи, понятные ответы по всем разделам анкеты
 • Чётко понимает свой график и готов регулярно помогать
-• Осознанная суперсила и понимание задач</t>
+• Осознанное понимание волонтёрских задач музея</t>
         </is>
       </c>
       <c r="D8" s="9" t="inlineStr">
@@ -1257,12 +1251,12 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>СТРОГО БУДНИ с 10:00 до 17:00–18:00 (хранилища закрыты по выходным)</t>
+          <t>Будние дни в дневное время (по согласованию с графиком хранителей отделов)</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>❌ КРАЙНЕ НИЗКАЯ для очников. Доступно выпускникам, вечерникам или при свободном посещении пар.</t>
+          <t>Требует индивидуальной проверки совпадения с учебным расписанием (свободные дни, вечернее отделение, индивидуальный график).</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
@@ -1272,7 +1266,7 @@
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>«Фонды работают только по будням с 10 до 18. Сможете ли вы присутствовать в эти часы без ущерба для учёбы?»</t>
+          <t>«Сможете ли вы участвовать в работе фондовых отделов в дневные часы по будням без ущерба для учёбы?»</t>
         </is>
       </c>
     </row>
@@ -1365,12 +1359,12 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Гибкий / удалённый график (с выездом на съёмки по согласованию)</t>
+          <t>Гибкий график: подготовка контента и очные выезды на съёмки мероприятий музея</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>✅ МАКСИМАЛЬНАЯ. Монтаж, тексты, дизайн и SMM можно выполнять дистанционно в удобное время.</t>
+          <t>Высокая при наличии навыков. Часть задач (дизайн, тексты) выполняется гибко, съёмки событий требуют очного присутствия в музее.</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
@@ -1442,7 +1436,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Утверждено заказчиком 21.10.2026: вопросы/ответы, баллы, саммари, возможные проблемы, рекомендуемое направление</t>
+          <t>Согласовано с представителем ГИМ 21.10.2026: вопросы/ответы, баллы (при наличии калиброванной шкалы), саммари, возможные проблемы, рекомендуемое направление.</t>
         </is>
       </c>
     </row>
@@ -1787,7 +1781,7 @@
     <row r="19">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>2. Точное рекомендуемое направление с учётом совместимости графика кандидата (например, очников не отправлять в будничные фонды).</t>
+          <t>2. Рекомендуемое направление с учётом графика кандидата (возможность участия в дневных сменах фондов согласовывать индивидуально).</t>
         </is>
       </c>
     </row>
@@ -1951,7 +1945,7 @@
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>Логический конфликт расписания (Hard Alert)</t>
+          <t>Проверяемая гипотеза графика (Alert)</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
@@ -1961,12 +1955,12 @@
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>Диалоговое предупреждение в форме: фонды работают строго в будни 10–18. Система предлагает переключиться на проекты/орг в выходные дни либо подтвердить свободное посещение.</t>
+          <t>Предупреждение: задачи фондов обычно проходят в дневные часы будних дней. Система предлагает подтвердить возможность участия в будни либо рассмотреть направления выходного дня (проекты/орг).</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>Оранжевый бейдж: «Конфликт расписания: очник претендует на фонды».</t>
+          <t>Оранжевый бейдж: «Уточнить график: очное обучение и задачи фондов».</t>
         </is>
       </c>
     </row>

</xml_diff>